<commit_message>
mantenimiento-preventivo: version HTML del cronograma y nombres de conjunto en espanol
Agrega la pagina HTML autonoma (resumen, agenda por cuadrilla, carga mensual,
detalle filtrable por casa, alertas y supuestos) y corrige las mayusculas de los
nombres de conjunto en el Excel (Reservas de Pance, Terra by Kaia, etc.).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0197ciwo2cQrNj8jqGbNoExn
</commit_message>
<xml_diff>
--- a/mantenimiento-preventivo/Cronograma_Mantenimiento_Preventivo_Sunny_2026-10.xlsx
+++ b/mantenimiento-preventivo/Cronograma_Mantenimiento_Preventivo_Sunny_2026-10.xlsx
@@ -83,13 +83,13 @@
     <t xml:space="preserve">Cali</t>
   </si>
   <si>
-    <t xml:space="preserve">Condominio Los Abedules; Llanos De Pance; Reservas De Pance</t>
+    <t xml:space="preserve">Condominio Los Abedules; Llanos de Pance; Reservas de Pance</t>
   </si>
   <si>
     <t xml:space="preserve">2, 10, 11, 12, 15, 18, 23, 29, 30, 35, 42, 48, 56, 57, 63, 70, 73, 74, 76, 77, 99, 104, 108, 111</t>
   </si>
   <si>
-    <t xml:space="preserve">Pance Campestre; Porton De La Rivera</t>
+    <t xml:space="preserve">Pance Campestre; Porton de la Rivera</t>
   </si>
   <si>
     <t xml:space="preserve">18PR, 48PC</t>
@@ -98,7 +98,7 @@
     <t xml:space="preserve">Costa</t>
   </si>
   <si>
-    <t xml:space="preserve">Prado Verde Primavera; Terra By Kaia</t>
+    <t xml:space="preserve">Prado Verde Primavera; Terra by Kaia</t>
   </si>
   <si>
     <t xml:space="preserve">18Ap, 23p, 24, 93p, 102p</t>
@@ -227,7 +227,7 @@
     <t xml:space="preserve">Sin histórico previo en Metrum; ya traía 2,61 MWh</t>
   </si>
   <si>
-    <t xml:space="preserve">Llanos De Pance</t>
+    <t xml:space="preserve">Llanos de Pance</t>
   </si>
   <si>
     <t xml:space="preserve">Casa 73</t>
@@ -239,7 +239,7 @@
     <t xml:space="preserve">Sin histórico previo en Metrum; ya traía 1,76 MWh</t>
   </si>
   <si>
-    <t xml:space="preserve">Reservas De Pance</t>
+    <t xml:space="preserve">Reservas de Pance</t>
   </si>
   <si>
     <t xml:space="preserve">Casa 2</t>
@@ -335,7 +335,7 @@
     <t xml:space="preserve">Costa - Atlántico</t>
   </si>
   <si>
-    <t xml:space="preserve">Terra By Kaia</t>
+    <t xml:space="preserve">Terra by Kaia</t>
   </si>
   <si>
     <t xml:space="preserve">Barranquilla</t>
@@ -494,7 +494,7 @@
     <t xml:space="preserve">Inversor reemplazado (equipo anterior sin datos desde 2026-08-22)</t>
   </si>
   <si>
-    <t xml:space="preserve">Porton De La Rivera</t>
+    <t xml:space="preserve">Porton de la Rivera</t>
   </si>
   <si>
     <t xml:space="preserve">Casa 18PR</t>

</xml_diff>